<commit_message>
chore: clean up old reports and fix cluster keywords; update metrics and test scripts for CVAE Flat
</commit_message>
<xml_diff>
--- a/data/results/p4_traditional_distinctive_it1000.xlsx
+++ b/data/results/p4_traditional_distinctive_it1000.xlsx
@@ -476,7 +476,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C965</t>
+          <t>pale</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -596,7 +596,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>C925</t>
+          <t>stove</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -626,7 +626,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C878</t>
+          <t>attention</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -636,7 +636,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>C945</t>
+          <t>woman</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -686,7 +686,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>C968</t>
+          <t>clothing</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -766,7 +766,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>C954</t>
+          <t>skills</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -886,7 +886,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>C461</t>
+          <t>buttocks</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -972,7 +972,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C969</t>
+          <t>grandchild</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1012,7 +1012,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C954</t>
+          <t>skills</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1042,7 +1042,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C957</t>
+          <t>collarbone</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1182,7 +1182,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>C977</t>
+          <t>income</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1302,7 +1302,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>C924</t>
+          <t>clothes</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1322,7 +1322,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>C942</t>
+          <t>eyebrows</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1382,7 +1382,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>C904</t>
+          <t>friend</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1462,7 +1462,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>C784</t>
+          <t>cigarette</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1518,7 +1518,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C994</t>
+          <t>fingertips</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1548,7 +1548,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C945</t>
+          <t>woman</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1578,7 +1578,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C957</t>
+          <t>collarbone</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1598,7 +1598,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C934</t>
+          <t>senior</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1668,7 +1668,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>C975</t>
+          <t>wrists</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1738,7 +1738,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>C965</t>
+          <t>pale</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1778,7 +1778,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>C627</t>
+          <t>son</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1808,7 +1808,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>C941</t>
+          <t>sister</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1818,7 +1818,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>C954</t>
+          <t>skills</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1938,7 +1938,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>C968</t>
+          <t>clothing</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1948,7 +1948,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>C903</t>
+          <t>money</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2084,7 +2084,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C965</t>
+          <t>pale</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2124,7 +2124,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C984</t>
+          <t>lucky</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2204,7 +2204,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C957</t>
+          <t>collarbone</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2254,7 +2254,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>C925</t>
+          <t>stove</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2294,7 +2294,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>C802</t>
+          <t>brother</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2304,7 +2304,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>C982</t>
+          <t>mouths</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2314,7 +2314,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>C968</t>
+          <t>clothing</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -2354,7 +2354,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>C966</t>
+          <t>able</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2404,7 +2404,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>C909</t>
+          <t>defloration</t>
         </is>
       </c>
       <c r="B40" t="n">

</xml_diff>